<commit_message>
Correct publication integrity controls
</commit_message>
<xml_diff>
--- a/AERA_1.2_WD_NIST_Mapping_Development_Ledger.xlsx
+++ b/AERA_1.2_WD_NIST_Mapping_Development_Ledger.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R6e24a390462047f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Ledger" sheetId="2" r:id="Reee8ef26c64046a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI RMF 1.0 Candidates" sheetId="3" r:id="R3c9e8fb27b2e4da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSF 2.0 Candidates" sheetId="4" r:id="R2b58f07de47f4d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP800-53 Candidates" sheetId="5" r:id="R6e3b2a32833744ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI RMF Design Attributes" sheetId="6" r:id="R793b4795ed48477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submission Checklist" sheetId="7" r:id="R3fc192d19e70481f"/>
-  </x:sheets>
-</x:workbook>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Read Me" sheetId="1" r:id="R62b38715a2aa4fbf"/>
+    <sheet name="Coverage Ledger" sheetId="2" r:id="R93446c32cbd6419e"/>
+    <sheet name="AI RMF 1.0 Candidates" sheetId="3" r:id="Rd55507e506194f8e"/>
+    <sheet name="CSF 2.0 Candidates" sheetId="4" r:id="R82b24e1acf7e430b"/>
+    <sheet name="SP800-53 Candidates" sheetId="5" r:id="R2e201d4cf1d84fe1"/>
+    <sheet name="AI RMF Design Attributes" sheetId="6" r:id="Rc8384cbfd9fc4761"/>
+    <sheet name="Submission Checklist" sheetId="7" r:id="R02665a4a6c844492"/>
+  </sheets>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -753,13 +754,13 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="19" t="str">
-        <x:v>Author / owner</x:v>
+        <x:v>Build ID</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>Angelis Pseftis / independent author</x:v>
+        <x:v>AERA-001-1.2WD-20260807.1</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>Named author and maintenance owner</x:v>
+        <x:v>Matches the controlled release manifest</x:v>
       </x:c>
       <x:c r="D6" s="18"/>
       <x:c r="E6" s="18"/>
@@ -769,13 +770,13 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="19" t="str">
-        <x:v>AERA requirements</x:v>
-      </x:c>
-      <x:c r="B7" s="18" t="n">
-        <x:v>199</x:v>
+        <x:v>Author / owner</x:v>
+      </x:c>
+      <x:c r="B7" s="18" t="str">
+        <x:v>Angelis Pseftis / independent author</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
-        <x:v>All requirements represented in Coverage Ledger</x:v>
+        <x:v>Named author and maintenance owner</x:v>
       </x:c>
       <x:c r="D7" s="18"/>
       <x:c r="E7" s="18"/>
@@ -785,13 +786,13 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="19" t="str">
-        <x:v>Mapping model</x:v>
+        <x:v>Public repository</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>NIST IR 8477 / IR 8278A Rev. 1</x:v>
+        <x:v>https://github.com/redxking/AERA</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>One atomic AERA-to-focal pair per assertion</x:v>
+        <x:v>Public snapshot published 2026-08-08; formal review not open</x:v>
       </x:c>
       <x:c r="D8" s="18"/>
       <x:c r="E8" s="18"/>
@@ -801,13 +802,13 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="19" t="str">
-        <x:v>Legacy D/P/E/C/N</x:v>
+        <x:v>Rights status</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>Preserved as unadjudicated source data</x:v>
+        <x:v>All rights reserved; no open license granted; contributions closed</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>No mechanical translation into IR 8477 relationships</x:v>
+        <x:v>No formal contribution or redistribution process is open</x:v>
       </x:c>
       <x:c r="D9" s="18"/>
       <x:c r="E9" s="18"/>
@@ -817,13 +818,13 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="19" t="str">
-        <x:v>OLIR status</x:v>
-      </x:c>
-      <x:c r="B10" s="18" t="str">
-        <x:v>NOT SUBMISSION READY</x:v>
+        <x:v>AERA requirements</x:v>
+      </x:c>
+      <x:c r="B10" s="18" t="n">
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>Exact target IDs/text, rationale, independent review and public artifacts complete</x:v>
+        <x:v>All requirements represented in Coverage Ledger</x:v>
       </x:c>
       <x:c r="D10" s="18"/>
       <x:c r="E10" s="18"/>
@@ -833,13 +834,13 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="19" t="str">
-        <x:v>Developmental review</x:v>
+        <x:v>Mapping model</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
-        <x:v>CANDIDATE - NOT OPEN</x:v>
+        <x:v>NIST IR 8477 / IR 8278A Rev. 1</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
-        <x:v>Stable URL or channel, dates, license, contribution and IP terms declared</x:v>
+        <x:v>One atomic AERA-to-focal pair per assertion</x:v>
       </x:c>
       <x:c r="D11" s="18"/>
       <x:c r="E11" s="18"/>
@@ -849,13 +850,13 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="19" t="str">
-        <x:v>NIST status</x:v>
+        <x:v>Legacy D/P/E/C/N</x:v>
       </x:c>
       <x:c r="B12" s="18" t="str">
-        <x:v>No review, support, acceptance or endorsement</x:v>
+        <x:v>Preserved as unadjudicated source data</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
-        <x:v>May change only with explicit documentary evidence</x:v>
+        <x:v>No mechanical translation into IR 8477 relationships</x:v>
       </x:c>
       <x:c r="D12" s="18"/>
       <x:c r="E12" s="18"/>
@@ -864,9 +865,15 @@
       <x:c r="H12" s="18"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="18"/>
-      <x:c r="B13" s="18"/>
-      <x:c r="C13" s="18"/>
+      <x:c r="A13" s="19" t="str">
+        <x:v>OLIR status</x:v>
+      </x:c>
+      <x:c r="B13" s="18" t="str">
+        <x:v>NOT SUBMISSION READY</x:v>
+      </x:c>
+      <x:c r="C13" s="18" t="str">
+        <x:v>Exact target IDs/text, rationale, independent review and public artifacts complete</x:v>
+      </x:c>
       <x:c r="D13" s="18"/>
       <x:c r="E13" s="18"/>
       <x:c r="F13" s="18"/>
@@ -874,118 +881,160 @@
       <x:c r="H13" s="18"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="20" t="str">
+      <x:c r="A14" s="19" t="str">
+        <x:v>Developmental review</x:v>
+      </x:c>
+      <x:c r="B14" s="18" t="str">
+        <x:v>PUBLIC SNAPSHOT; FORMAL REVIEW NOT OPEN</x:v>
+      </x:c>
+      <x:c r="C14" s="18" t="str">
+        <x:v>Formal channel, dates, contribution/IP, privacy and moderation terms declared</x:v>
+      </x:c>
+      <x:c r="D14" s="18"/>
+      <x:c r="E14" s="18"/>
+      <x:c r="F14" s="18"/>
+      <x:c r="G14" s="18"/>
+      <x:c r="H14" s="18"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="19" t="str">
+        <x:v>NIST status</x:v>
+      </x:c>
+      <x:c r="B15" s="18" t="str">
+        <x:v>No review, support, acceptance or endorsement</x:v>
+      </x:c>
+      <x:c r="C15" s="18" t="str">
+        <x:v>May change only with explicit documentary evidence</x:v>
+      </x:c>
+      <x:c r="D15" s="18"/>
+      <x:c r="E15" s="18"/>
+      <x:c r="F15" s="18"/>
+      <x:c r="G15" s="18"/>
+      <x:c r="H15" s="18"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="18"/>
+      <x:c r="B16" s="18"/>
+      <x:c r="C16" s="18"/>
+      <x:c r="D16" s="18"/>
+      <x:c r="E16" s="18"/>
+      <x:c r="F16" s="18"/>
+      <x:c r="G16" s="18"/>
+      <x:c r="H16" s="18"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="20" t="str">
         <x:v>Mapping lanes</x:v>
       </x:c>
-      <x:c r="B14" s="20"/>
-      <x:c r="C14" s="20"/>
-      <x:c r="D14" s="20"/>
-      <x:c r="E14" s="20"/>
-      <x:c r="F14" s="20"/>
-      <x:c r="G14" s="20"/>
-      <x:c r="H14" s="20"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="16" t="str">
+      <x:c r="B17" s="20"/>
+      <x:c r="C17" s="20"/>
+      <x:c r="D17" s="20"/>
+      <x:c r="E17" s="20"/>
+      <x:c r="F17" s="20"/>
+      <x:c r="G17" s="20"/>
+      <x:c r="H17" s="20"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="16" t="str">
         <x:v>Lane</x:v>
       </x:c>
-      <x:c r="B15" s="16" t="str">
+      <x:c r="B18" s="16" t="str">
         <x:v>Focal document</x:v>
       </x:c>
-      <x:c r="C15" s="16" t="str">
+      <x:c r="C18" s="16" t="str">
         <x:v>Relationship style</x:v>
       </x:c>
-      <x:c r="D15" s="16" t="str">
+      <x:c r="D18" s="16" t="str">
         <x:v>Current state</x:v>
       </x:c>
-      <x:c r="E15" s="16" t="str">
+      <x:c r="E18" s="16" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="F15" s="16" t="str">
+      <x:c r="F18" s="16" t="str">
         <x:v>Independent reviewer</x:v>
       </x:c>
-      <x:c r="G15" s="16" t="str">
+      <x:c r="G18" s="16" t="str">
         <x:v>Developmental review</x:v>
       </x:c>
-      <x:c r="H15" s="16" t="str">
+      <x:c r="H18" s="16" t="str">
         <x:v>Maintenance</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="18" t="str">
+    <x:row r="19">
+      <x:c r="A19" s="18" t="str">
         <x:v>AI RMF</x:v>
       </x:c>
-      <x:c r="B16" s="18" t="str">
+      <x:c r="B19" s="18" t="str">
         <x:v>NIST AI RMF 1.0</x:v>
       </x:c>
-      <x:c r="C16" s="18" t="str">
+      <x:c r="C19" s="18" t="str">
         <x:v>Supportive mapping candidate</x:v>
       </x:c>
-      <x:c r="D16" s="18" t="str">
+      <x:c r="D19" s="18" t="str">
         <x:v>Screening only</x:v>
       </x:c>
-      <x:c r="E16" s="18" t="str">
+      <x:c r="E19" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="F16" s="18" t="str">
+      <x:c r="F19" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="G16" s="18" t="str">
+      <x:c r="G19" s="18" t="str">
         <x:v>CANDIDATE - NOT OPEN</x:v>
       </x:c>
-      <x:c r="H16" s="18" t="str">
+      <x:c r="H19" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="18" t="str">
+    <x:row r="20">
+      <x:c r="A20" s="18" t="str">
         <x:v>CSF</x:v>
       </x:c>
-      <x:c r="B17" s="18" t="str">
+      <x:c r="B20" s="18" t="str">
         <x:v>NIST CSF 2.0</x:v>
       </x:c>
-      <x:c r="C17" s="18" t="str">
+      <x:c r="C20" s="18" t="str">
         <x:v>Supportive mapping candidate</x:v>
       </x:c>
-      <x:c r="D17" s="18" t="str">
+      <x:c r="D20" s="18" t="str">
         <x:v>Screening only</x:v>
       </x:c>
-      <x:c r="E17" s="18" t="str">
+      <x:c r="E20" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="F17" s="18" t="str">
+      <x:c r="F20" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="G17" s="18" t="str">
+      <x:c r="G20" s="18" t="str">
         <x:v>CANDIDATE - NOT OPEN</x:v>
       </x:c>
-      <x:c r="H17" s="18" t="str">
+      <x:c r="H20" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="18" t="str">
+    <x:row r="21">
+      <x:c r="A21" s="18" t="str">
         <x:v>SP 800-53</x:v>
       </x:c>
-      <x:c r="B18" s="18" t="str">
+      <x:c r="B21" s="18" t="str">
         <x:v>SP 800-53 Rev. 5 Release 5.2.0</x:v>
       </x:c>
-      <x:c r="C18" s="18" t="str">
+      <x:c r="C21" s="18" t="str">
         <x:v>Supportive or concept mapping candidate</x:v>
       </x:c>
-      <x:c r="D18" s="18" t="str">
+      <x:c r="D21" s="18" t="str">
         <x:v>Screening only</x:v>
       </x:c>
-      <x:c r="E18" s="18" t="str">
+      <x:c r="E21" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="F18" s="18" t="str">
+      <x:c r="F21" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
-      <x:c r="G18" s="18" t="str">
+      <x:c r="G21" s="18" t="str">
         <x:v>CANDIDATE - NOT OPEN</x:v>
       </x:c>
-      <x:c r="H18" s="18" t="str">
+      <x:c r="H21" s="18" t="str">
         <x:v>OPEN</x:v>
       </x:c>
     </x:row>
@@ -993,7 +1042,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A14:H14"/>
+    <x:mergeCell ref="A17:H17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8644,7 +8693,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4748d81048164f6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R566c39434ea448c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11056,7 +11105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb793b4b05c2463c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re27288380213457b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14092,7 +14141,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cc07a7d8def4666"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R652dbb434aa14185"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17986,7 +18035,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcc0d173427948b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R965b3332d40148c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18158,7 +18207,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f1cfe7059034e7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf61d5068e6154691"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18203,12 +18252,16 @@
         <x:v>Stable public AERA document and mapping URLs</x:v>
       </x:c>
       <x:c r="C2" s="44" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="D2" s="44"/>
-      <x:c r="E2" s="44"/>
+        <x:v>COMPLETE</x:v>
+      </x:c>
+      <x:c r="D2" s="44" t="str">
+        <x:v>Angelis Pseftis</x:v>
+      </x:c>
+      <x:c r="E2" s="44" t="str">
+        <x:v>https://github.com/redxking/AERA</x:v>
+      </x:c>
       <x:c r="F2" s="45" t="str">
-        <x:v>No public release verified</x:v>
+        <x:v>Public snapshot verified; formal public review remains closed</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="62" customHeight="1">
@@ -18219,12 +18272,16 @@
         <x:v>Declared license, contribution terms and IP process</x:v>
       </x:c>
       <x:c r="C3" s="44" t="str">
-        <x:v>OPEN - AUTHOR DECISION</x:v>
-      </x:c>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="D3" s="44" t="str">
+        <x:v>Angelis Pseftis</x:v>
+      </x:c>
+      <x:c r="E3" s="44" t="str">
+        <x:v>LICENSE.md; CONTRIBUTING.md</x:v>
+      </x:c>
       <x:c r="F3" s="45" t="str">
-        <x:v>Required before public redistribution or submission</x:v>
+        <x:v>No open license or formal contribution/IP process; not ready for formal review or submission</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
@@ -18365,7 +18422,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7b778278f8d4c29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb613cd60100f4842"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>